<commit_message>
scan: seg5 2026-07-10 18:58 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq6_2026-07-09.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1156.488689421495</v>
+        <v>1136.488689421495</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>73.3</v>
@@ -633,21 +633,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>6214</v>
+        <v>6416</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>精誠</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>999.071936332872</v>
+        <v>979.3786316376716</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>143.5</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>60.50422918684576</v>
+        <v>76.06429831862002</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>17.0889865435334</v>
+        <v>25.63228320159281</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2.433126022514748</v>
+        <v>3.537863163767159</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -676,31 +676,31 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.3179615362093037</v>
+        <v>2.003064935013459</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, cci_momentum, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>6416</v>
+        <v>6257</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>979.3786316376716</v>
+        <v>961.4087282385286</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>244.5</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,49 +711,49 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>76.06429831862002</v>
+        <v>55.05093771502047</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>25.63228320159281</v>
+        <v>23.26007460439195</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>3.537863163767159</v>
+        <v>0.5128257206867946</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>2.003064935013459</v>
+        <v>0.3007865075158751</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>6257</v>
+        <v>6214</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>精誠</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>961.4087282385286</v>
+        <v>959.0719363328718</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>244.5</v>
+        <v>143.5</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,29 +764,29 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.05093771502047</v>
+        <v>60.50422918684576</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23.26007460439195</v>
+        <v>17.0889865435334</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.5128257206867946</v>
+        <v>2.433126022514748</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.3007865075158751</v>
+        <v>0.3179615362093037</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, cci_momentum, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -845,41 +845,41 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6288</v>
+        <v>6226</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>聯嘉</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>933.7637113435804</v>
+        <v>935.8896455488092</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>24.25</v>
+        <v>26.6</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G8" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>66.26037974163694</v>
+        <v>76.94869745174736</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>25.42428002621412</v>
+        <v>38.68939568950388</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>3.476371134358034</v>
+        <v>0.5810445043913632</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -888,64 +888,64 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.2001952343977984</v>
+        <v>0.8074758270968085</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6213</v>
+        <v>6288</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>聯茂</t>
+          <t>聯嘉</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>918.2917432855902</v>
+        <v>933.7637113435804</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>385</v>
+        <v>24.25</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="G9" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66.52584889707384</v>
+        <v>66.26037974163694</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>27.52381890203836</v>
+        <v>25.42428002621412</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.258419360207691</v>
+        <v>3.476371134358034</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>5.515810684032736</v>
+        <v>0.2001952343977984</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1057,21 +1057,21 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6197</v>
+        <v>6213</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>佳必琪</t>
+          <t>聯茂</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>828.220035793717</v>
+        <v>878.2917432855902</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>358.5</v>
+        <v>385</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,29 +1082,29 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.69446535738361</v>
+        <v>66.52584889707384</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>40.89797096720127</v>
+        <v>27.52381890203836</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.8309268861561855</v>
+        <v>1.258419360207691</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-3.042639085888481</v>
+        <v>5.515810684032736</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1269,21 +1269,21 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6474</v>
+        <v>6197</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>華豫寧</t>
+          <t>佳必琪</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>784.2051585237849</v>
+        <v>788.220035793717</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>38.75</v>
+        <v>358.5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,49 +1294,49 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53.57639518225029</v>
+        <v>58.69446535738361</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>12.80507530958565</v>
+        <v>40.89797096720127</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2.534434889060984</v>
+        <v>0.8309268861561855</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.2731071982135357</v>
+        <v>-3.042639085888481</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6446</v>
+        <v>6474</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>華豫寧</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>769.0145008508529</v>
+        <v>784.2051585237849</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1285</v>
+        <v>38.75</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.93346557721873</v>
+        <v>53.57639518225029</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>55.03703858800521</v>
+        <v>12.80507530958565</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>2.119483154784996</v>
+        <v>2.534434889060984</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>10.00340540925461</v>
+        <v>0.2731071982135357</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>6418</v>
+        <v>6446</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>詠昇</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>746.6754752259185</v>
+        <v>769.0145008508529</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>33.45</v>
+        <v>1285</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,16 +1400,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>56.48690536370351</v>
+        <v>57.93346557721873</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>22.87147165554896</v>
+        <v>55.03703858800521</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.4200120058314038</v>
+        <v>2.119483154784996</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.2339394278810898</v>
+        <v>10.00340540925461</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6209</v>
+        <v>6418</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>詠昇</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>743.8443291860746</v>
+        <v>746.6754752259185</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>80.8</v>
+        <v>33.45</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>48.67482667949162</v>
+        <v>56.48690536370351</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>26.55887681155335</v>
+        <v>22.87147165554896</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0.4540819283646607</v>
+        <v>0.4200120058314038</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>0</v>
@@ -1471,11 +1471,11 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-1.372872544755097</v>
+        <v>0.2339394278810898</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1693,21 +1693,21 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6464</v>
+        <v>6209</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>台數科</t>
+          <t>今國光</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>695.2697929953064</v>
+        <v>703.8443291860746</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>77.59999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,13 +1718,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>48.90657935374674</v>
+        <v>48.67482667949162</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>25.09064688837675</v>
+        <v>26.55887681155335</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>2.342905295017971</v>
+        <v>0.4540819283646607</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>2</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.0234452478394544</v>
+        <v>-1.372872544755097</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6265</v>
+        <v>6464</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>方土昶</t>
+          <t>台數科</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>692.3907045959453</v>
+        <v>695.2697929953064</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>52.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>49.41435432158837</v>
+        <v>48.90657935374674</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>18.56809377486853</v>
+        <v>25.09064688837675</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.7408096669763091</v>
+        <v>2.342905295017971</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.6597679191502358</v>
+        <v>-0.0234452478394544</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6279</v>
+        <v>6265</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>胡連</t>
+          <t>方土昶</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>690.7722923356679</v>
+        <v>692.3907045959453</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>122.5</v>
+        <v>52.7</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>56.80840944499453</v>
+        <v>49.41435432158837</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>19.39694305229023</v>
+        <v>18.56809377486853</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.8675874942786891</v>
+        <v>0.7408096669763091</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.3843443813994877</v>
+        <v>-0.6597679191502358</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6409</v>
+        <v>6279</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>旭隼</t>
+          <t>胡連</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>660.6657833783099</v>
+        <v>690.7722923356679</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1105</v>
+        <v>122.5</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>58.79025671788048</v>
+        <v>56.80840944499453</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>49.21872680775778</v>
+        <v>19.39694305229023</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.5077861502365508</v>
+        <v>0.8675874942786891</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>6.427115661867504</v>
+        <v>0.3843443813994877</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6246</v>
+        <v>6409</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>臺龍</t>
+          <t>旭隼</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>646.7553999006445</v>
+        <v>660.6657833783099</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>15.4</v>
+        <v>1105</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46.68802759221125</v>
+        <v>58.79025671788048</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21.59670668951503</v>
+        <v>49.21872680775778</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.298702357410885</v>
+        <v>0.5077861502365508</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.0424925612897447</v>
+        <v>6.427115661867504</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6419</v>
+        <v>6246</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>京晨科</t>
+          <t>臺龍</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>637.2875668941255</v>
+        <v>646.7553999006445</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>146</v>
+        <v>15.4</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.10961573079987</v>
+        <v>46.68802759221125</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>9.233091069412589</v>
+        <v>21.59670668951503</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.4496120911036987</v>
+        <v>0.298702357410885</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.1655321847692704</v>
+        <v>-0.0424925612897447</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6175</v>
+        <v>6419</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>京晨科</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>630.7023836445761</v>
+        <v>637.2875668941255</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.64811739707996</v>
+        <v>51.10961573079987</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>35.94163140743942</v>
+        <v>9.233091069412589</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.3016672626794371</v>
+        <v>0.4496120911036987</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-1.732389440968922</v>
+        <v>-0.1655321847692704</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6271</v>
+        <v>6176</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>621.0928621229963</v>
+        <v>630.7227281970102</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>252</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>51.19847872710957</v>
+        <v>45.95921703984428</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.45229549813269</v>
+        <v>18.23336187973892</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.5346225556122013</v>
+        <v>0.4865562411329991</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-2.368416313269387</v>
+        <v>0.7301936113755336</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6187</v>
+        <v>6175</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>萬潤</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>612.8943797335932</v>
+        <v>630.7023836445761</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1050</v>
+        <v>105</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,49 +2142,49 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.66755686619767</v>
+        <v>50.64811739707996</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>10.93429019971599</v>
+        <v>35.94163140743942</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.418708493139663</v>
+        <v>0.3016672626794371</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M32" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-8.324338563349585</v>
+        <v>-1.732389440968922</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6204</v>
+        <v>6271</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>艾華</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>604.8897832036441</v>
+        <v>621.0928621229963</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>98.5</v>
+        <v>252</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>41.48366736939177</v>
+        <v>51.19847872710957</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>28.33411598523973</v>
+        <v>24.45229549813269</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.4866331027247718</v>
+        <v>0.5346225556122013</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-3.300467962525275</v>
+        <v>-2.368416313269387</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6196</v>
+        <v>6187</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>萬潤</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>600.7545257562992</v>
+        <v>612.8943797335932</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>549</v>
+        <v>1050</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,49 +2248,49 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.08532215887169</v>
+        <v>48.66755686619767</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>28.05357859083168</v>
+        <v>10.93429019971599</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.8671349625130681</v>
+        <v>1.418708493139663</v>
       </c>
       <c r="K34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L34" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M34" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-5.07453997068513</v>
+        <v>-8.324338563349585</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6176</v>
+        <v>6204</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>艾華</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>600.7227281970102</v>
+        <v>604.8897832036441</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>90.59999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>45.95921703984428</v>
+        <v>41.48366736939177</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>18.23336187973892</v>
+        <v>28.33411598523973</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.4865562411329991</v>
+        <v>0.4866331027247718</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,11 +2319,11 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.7301936113755336</v>
+        <v>-3.300467962525275</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6166</v>
+        <v>6435</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>凌華</t>
+          <t>大中</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>589.6703293062818</v>
+        <v>576.1851267043151</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>134.5</v>
+        <v>375</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>50.95900459453849</v>
+        <v>60.02396593640601</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>37.25304903070406</v>
+        <v>35.11373582234368</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.6481348291603305</v>
+        <v>0.800487862173044</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-2.634043287392596</v>
+        <v>1.27326385425064</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6165</v>
+        <v>6465</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>威潤</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>589.5856464879407</v>
+        <v>575.1809853817028</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>50.1</v>
+        <v>63.3</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>55.89803805348778</v>
+        <v>56.1046732562139</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>20.28593810246351</v>
+        <v>26.27029971801192</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.049333799631696</v>
+        <v>0.753080817871749</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.3791670455581503</v>
+        <v>-1.136157175014425</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6435</v>
+        <v>6208</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>大中</t>
+          <t>日揚</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>576.1851267043151</v>
+        <v>574.229836358609</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>375</v>
+        <v>90.3</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>60.02396593640601</v>
+        <v>47.39148571270285</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>35.11373582234368</v>
+        <v>15.45204016428327</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.800487862173044</v>
+        <v>0.1722180031841522</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>1.27326385425064</v>
+        <v>-1.225666944879956</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6465</v>
+        <v>6239</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>威潤</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>575.1809853817028</v>
+        <v>573.9125542434286</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>63.3</v>
+        <v>320</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,49 +2937,49 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>56.1046732562139</v>
+        <v>48.44503578764906</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>26.27029971801192</v>
+        <v>23.80075786039455</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.753080817871749</v>
+        <v>0.3459569826215111</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M47" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-1.136157175014425</v>
+        <v>-4.586864459811611</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6208</v>
+        <v>6165</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>日揚</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>574.229836358609</v>
+        <v>569.5856464879407</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>90.3</v>
+        <v>50.1</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>47.39148571270285</v>
+        <v>55.89803805348778</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>15.45204016428327</v>
+        <v>20.28593810246351</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.1722180031841522</v>
+        <v>1.049333799631696</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.225666944879956</v>
+        <v>0.3791670455581503</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6239</v>
+        <v>6235</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>華孚</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>573.9125542434286</v>
+        <v>564.7068725170659</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>320</v>
+        <v>42.4</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,49 +3043,49 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>48.44503578764906</v>
+        <v>50.95768947600303</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.80075786039455</v>
+        <v>20.46692171898411</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.3459569826215111</v>
+        <v>1.042148858262224</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-4.586864459811611</v>
+        <v>0.4104142795117735</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6235</v>
+        <v>6196</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>華孚</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>564.7068725170659</v>
+        <v>560.7545257562992</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>42.4</v>
+        <v>549</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>50.95768947600303</v>
+        <v>54.08532215887169</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>20.46692171898411</v>
+        <v>28.05357859083168</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.042148858262224</v>
+        <v>0.8671349625130681</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.4104142795117735</v>
+        <v>-5.07453997068513</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6206</v>
+        <v>6166</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>飛捷</t>
+          <t>凌華</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>557.206889349207</v>
+        <v>549.6703293062818</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>131.5</v>
+        <v>134.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>50.80161092657132</v>
+        <v>50.95900459453849</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>11.05857041742693</v>
+        <v>37.25304903070406</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.596155571684044</v>
+        <v>0.6481348291603305</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,11 +3167,11 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.1683190083713577</v>
+        <v>-2.634043287392596</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3230,21 +3230,21 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6189</v>
+        <v>6261</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>豐藝</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>543.1171308580567</v>
+        <v>539.7984202187615</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>50.4</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>44.42019512273473</v>
+        <v>39.89966499434699</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.72534459086502</v>
+        <v>17.70217002504111</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.2994648258745055</v>
+        <v>0.3258076319138756</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.32970209837375</v>
+        <v>-0.0227109598430041</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6261</v>
+        <v>6173</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>信昌電</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>539.7984202187615</v>
+        <v>526.9722281302035</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>275</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>39.89966499434699</v>
+        <v>50.18098418175746</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>17.70217002504111</v>
+        <v>26.82029344258599</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3258076319138756</v>
+        <v>1.056435950495918</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.0227109598430041</v>
+        <v>-8.545329832583654</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6215</v>
+        <v>6189</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>和椿</t>
+          <t>豐藝</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>528.0668217122557</v>
+        <v>523.1171308580568</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>113.5</v>
+        <v>50.4</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>51.95973173451051</v>
+        <v>44.42019512273473</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>17.62415730350409</v>
+        <v>18.72534459086502</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.944676363510302</v>
+        <v>0.2994648258745055</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.398526045593522</v>
+        <v>-0.32970209837375</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6173</v>
+        <v>6192</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>信昌電</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>526.9722281302035</v>
+        <v>522.7966888452497</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>275</v>
+        <v>120</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>50.18098418175746</v>
+        <v>46.57038285186782</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>26.82029344258599</v>
+        <v>19.77975771667846</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.056435950495918</v>
+        <v>0.2885966311380484</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-8.545329832583654</v>
+        <v>0.1031038247129059</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6228</v>
+        <v>6206</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>全譜</t>
+          <t>飛捷</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>505.2527726489098</v>
+        <v>517.206889349207</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>19.1</v>
+        <v>131.5</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>44.66734659846346</v>
+        <v>50.80161092657132</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>4.744489874638209</v>
+        <v>11.05857041742693</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.1213040586205195</v>
+        <v>1.596155571684044</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.0666148916581248</v>
+        <v>0.1683190083713577</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6244</v>
+        <v>6216</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>茂迪</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>503.2552975876344</v>
+        <v>509.7726759338609</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>27</v>
+        <v>23.15</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>45.56871279071334</v>
+        <v>52.51581439552675</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>10.21266174976934</v>
+        <v>12.02130481601512</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.2920367732268786</v>
+        <v>0.6623511287610836</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.0648959710707384</v>
+        <v>0.05811366871442</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6277</v>
+        <v>6228</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>宏正</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>498.0865178878039</v>
+        <v>505.2527726489098</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>70.7</v>
+        <v>19.1</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.52558862040208</v>
+        <v>44.66734659846346</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>26.28544254631901</v>
+        <v>4.744489874638209</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.6633441183231713</v>
+        <v>0.1213040586205195</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0103847418663265</v>
+        <v>-0.0666148916581248</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6192</v>
+        <v>6244</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>茂迪</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>492.7966888452498</v>
+        <v>503.2552975876344</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>120</v>
+        <v>27</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46.57038285186782</v>
+        <v>45.56871279071334</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>19.77975771667846</v>
+        <v>10.21266174976934</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.2885966311380484</v>
+        <v>0.2920367732268786</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.1031038247129059</v>
+        <v>-0.0648959710707384</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6263</v>
+        <v>6277</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>普萊德</t>
+          <t>宏正</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>489.8567207262365</v>
+        <v>498.0865178878039</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>167</v>
+        <v>70.7</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.75347187899839</v>
+        <v>44.52558862040208</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>12.24218822397629</v>
+        <v>26.28544254631901</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.5858107371423468</v>
+        <v>0.6633441183231713</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.583381093773764</v>
+        <v>-0.0103847418663265</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6216</v>
+        <v>6263</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>普萊德</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>479.7726759338609</v>
+        <v>489.8567207262365</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>23.15</v>
+        <v>167</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>52.51581439552675</v>
+        <v>51.75347187899839</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>12.02130481601512</v>
+        <v>12.24218822397629</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.6623511287610836</v>
+        <v>0.5858107371423468</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.05811366871442</v>
+        <v>0.583381093773764</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6275</v>
+        <v>6215</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>元山</t>
+          <t>和椿</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>473.4980509542552</v>
+        <v>488.0668217122557</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>48.1</v>
+        <v>113.5</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.3304117156073</v>
+        <v>51.95973173451051</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>11.7577176448209</v>
+        <v>17.62415730350409</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.2776469834185253</v>
+        <v>0.944676363510302</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.09199118072810079</v>
+        <v>1.398526045593522</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6210</v>
+        <v>6275</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>慶生</t>
+          <t>元山</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>464.6667525024073</v>
+        <v>473.4980509542552</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>19.75</v>
+        <v>48.1</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>42.44888140220458</v>
+        <v>45.3304117156073</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>23.62073255125464</v>
+        <v>11.7577176448209</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.2857534482077683</v>
+        <v>0.2776469834185253</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.0988259565309022</v>
+        <v>-0.09199118072810079</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6168</v>
+        <v>6210</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>宏齊</t>
+          <t>慶生</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>463.7828326677232</v>
+        <v>464.6667525024073</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>28.85</v>
+        <v>19.75</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>48.91567536944652</v>
+        <v>42.44888140220458</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>23.86009076031464</v>
+        <v>23.62073255125464</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.5031973367918018</v>
+        <v>0.2857534482077683</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,11 +3909,11 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.2869513207650043</v>
+        <v>-0.0988259565309022</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -4237,21 +4237,21 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6292</v>
+        <v>6168</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>迅德</t>
+          <t>宏齊</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>442.7728954449452</v>
+        <v>443.7828326677232</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>58.1</v>
+        <v>28.85</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>45.35527093712343</v>
+        <v>48.91567536944652</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.68220543669655</v>
+        <v>23.86009076031464</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.2143510663185322</v>
+        <v>0.5031973367918018</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.8259917223017678</v>
+        <v>-0.2869513207650043</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6426</v>
+        <v>6292</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>統新</t>
+          <t>迅德</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>437.8548021120627</v>
+        <v>442.7728954449452</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>187.5</v>
+        <v>58.1</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>40.50472524134657</v>
+        <v>45.35527093712343</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>17.42581142994613</v>
+        <v>22.68220543669655</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.5711687107957454</v>
+        <v>0.2143510663185322</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.238914626899529</v>
+        <v>-0.8259917223017678</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6470</v>
+        <v>6426</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>宇智</t>
+          <t>統新</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>428.6954580025336</v>
+        <v>437.8548021120627</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>48.2</v>
+        <v>187.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>43.87120259228157</v>
+        <v>40.50472524134657</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>10.7933361805923</v>
+        <v>17.42581142994613</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2870718049139532</v>
+        <v>0.5711687107957454</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.1652794096263817</v>
+        <v>-0.238914626899529</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6177</v>
+        <v>6201</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>達麗</t>
+          <t>亞弘電</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>425.9484505658648</v>
+        <v>429.3913444803261</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>45.3</v>
+        <v>48.2</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>47.57489387764495</v>
+        <v>47.25179204900812</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>18.49489665722346</v>
+        <v>12.91561406465129</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.2200969188721565</v>
+        <v>0.7091451287235034</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.1489141335302252</v>
+        <v>0.07570005957403431</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6237</v>
+        <v>6470</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>宇智</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>424.5636897177679</v>
+        <v>428.6954580025336</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>42</v>
+        <v>48.2</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.47391672999221</v>
+        <v>43.87120259228157</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>15.33426235374559</v>
+        <v>10.7933361805923</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.3681852680468525</v>
+        <v>0.2870718049139532</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.4402223312269442</v>
+        <v>-0.1652794096263817</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6218</v>
+        <v>6177</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>達麗</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>423.5998250586194</v>
+        <v>425.9484505658648</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>37.65</v>
+        <v>45.3</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>53.71863566754495</v>
+        <v>47.57489387764495</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>12.11336053714617</v>
+        <v>18.49489665722346</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.7799099700886115</v>
+        <v>0.2200969188721565</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.0765627468007149</v>
+        <v>-0.1489141335302252</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6438</v>
+        <v>6237</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>420.9571224619286</v>
+        <v>424.5636897177679</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>150</v>
+        <v>42</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.43657643210879</v>
+        <v>39.47391672999221</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.95269682823951</v>
+        <v>15.33426235374559</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.355053965030203</v>
+        <v>0.3681852680468525</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.0937697190638255</v>
+        <v>-0.4402223312269442</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6184</v>
+        <v>6218</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>大豐電</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>420.1887932823112</v>
+        <v>423.5998250586194</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>42.95</v>
+        <v>37.65</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>23.08460877876179</v>
+        <v>53.71863566754495</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>34.84741265862615</v>
+        <v>12.11336053714617</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.3583230749555412</v>
+        <v>0.7799099700886115</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.164233773995498</v>
+        <v>-0.0765627468007149</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6190</v>
+        <v>6438</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>418.9408680563363</v>
+        <v>420.9571224619286</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>82.09999999999999</v>
+        <v>150</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>50.34237102418618</v>
+        <v>42.43657643210879</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>15.63189548975667</v>
+        <v>18.95269682823951</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.4859050337067814</v>
+        <v>0.355053965030203</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.2071625297881087</v>
+        <v>0.0937697190638255</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6167</v>
+        <v>6184</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>大豐電</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>418.1672673971372</v>
+        <v>420.1887932823112</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>11.95</v>
+        <v>42.95</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>48.06859488036503</v>
+        <v>23.08460877876179</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>12.51517199083887</v>
+        <v>34.84741265862615</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.3064617242987439</v>
+        <v>0.3583230749555412</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-3.267974353826641e-05</v>
+        <v>-0.164233773995498</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6191</v>
+        <v>6190</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>417.6157292145597</v>
+        <v>418.9408680563363</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>101</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>48.80069786817602</v>
+        <v>50.34237102418618</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.93277159754891</v>
+        <v>15.63189548975667</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.4765533747053406</v>
+        <v>0.4859050337067814</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0634150839392706</v>
+        <v>-0.2071625297881087</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6198</v>
+        <v>6167</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>410.9554246216042</v>
+        <v>418.1672673971372</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>20.35</v>
+        <v>11.95</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>50.12740667423494</v>
+        <v>48.06859488036503</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>7.069923903668688</v>
+        <v>12.51517199083887</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.4026442608430207</v>
+        <v>0.3064617242987439</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0011358756227049</v>
+        <v>-3.267974353826641e-05</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6291</v>
+        <v>6191</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>405.8446327600136</v>
+        <v>417.6157292145597</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>463.5</v>
+        <v>101</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,49 +4898,49 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.12907838236885</v>
+        <v>48.80069786817602</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>15.65361422755754</v>
+        <v>27.93277159754891</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.6961864646384438</v>
+        <v>0.4765533747053406</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-15.20329251158969</v>
+        <v>-0.0634150839392706</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6278</v>
+        <v>6198</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>瑞築</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>404.0760437863103</v>
+        <v>410.9554246216042</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>199.5</v>
+        <v>20.35</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,49 +4951,49 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.86320449976485</v>
+        <v>50.12740667423494</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>16.013163606553</v>
+        <v>7.069923903668688</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.9402907544968636</v>
+        <v>0.4026442608430207</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.130259753047042</v>
+        <v>0.0011358756227049</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6225</v>
+        <v>6291</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>天瀚</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>402.9006456083451</v>
+        <v>405.8446327600136</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>23.3</v>
+        <v>463.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,49 +5004,49 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>51.86622281759339</v>
+        <v>40.12907838236885</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>11.41918567163419</v>
+        <v>15.65361422755754</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.2609126346787915</v>
+        <v>0.6961864646384438</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M86" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.2546357645545872</v>
+        <v>-15.20329251158969</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6188</v>
+        <v>6278</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>400.8744673379965</v>
+        <v>404.0760437863103</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>78.5</v>
+        <v>199.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,49 +5057,49 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>46.19150541009052</v>
+        <v>47.86320449976485</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>12.25889404109576</v>
+        <v>16.013163606553</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.2737012737776226</v>
+        <v>0.9402907544968636</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M87" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.3939372098629272</v>
+        <v>-1.130259753047042</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6201</v>
+        <v>6188</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>廣明</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>399.3913444803261</v>
+        <v>400.8744673379965</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>48.2</v>
+        <v>78.5</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>47.25179204900812</v>
+        <v>46.19150541009052</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>12.91561406465129</v>
+        <v>12.25889404109576</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.7091451287235034</v>
+        <v>0.2737012737776226</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.07570005957403431</v>
+        <v>0.3939372098629272</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6227</v>
+        <v>6164</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>茂綸</t>
+          <t>華興</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>383.3636657148558</v>
+        <v>389.9481550569465</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>120.5</v>
+        <v>14.95</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>48.45918465624463</v>
+        <v>56.66915190676168</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>12.12125093120201</v>
+        <v>25.98464873145076</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5060957319090983</v>
+        <v>0.8948155056946507</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.4692695135204854</v>
+        <v>0.1312034857149905</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6284</v>
+        <v>6227</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>佳邦</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>382.1485316065958</v>
+        <v>383.3636657148558</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>99.5</v>
+        <v>120.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>47.79353147360386</v>
+        <v>48.45918465624463</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>30.75634827810249</v>
+        <v>12.12125093120201</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.6125609446353782</v>
+        <v>0.5060957319090983</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.579809785626451</v>
+        <v>-0.4692695135204854</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6272</v>
+        <v>6284</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>驊陞</t>
+          <t>佳邦</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>378.669402588067</v>
+        <v>382.1485316065958</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>31.45</v>
+        <v>99.5</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>43.6264995451436</v>
+        <v>47.79353147360386</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>17.96242195034485</v>
+        <v>30.75634827810249</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.5504062374758626</v>
+        <v>0.6125609446353782</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.0261488976026397</v>
+        <v>-0.579809785626451</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6229</v>
+        <v>6272</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>研通</t>
+          <t>驊陞</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>377.5814319377752</v>
+        <v>378.669402588067</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>26.2</v>
+        <v>31.45</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>44.35274045183917</v>
+        <v>43.6264995451436</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>9.892033945605846</v>
+        <v>17.96242195034485</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.2346939174278734</v>
+        <v>0.5504062374758626</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.1126878788656517</v>
+        <v>-0.0261488976026397</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6442</v>
+        <v>6229</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>研通</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>372.1757267281355</v>
+        <v>377.5814319377752</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>1480</v>
+        <v>26.2</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,49 +5375,49 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.11839568595813</v>
+        <v>44.35274045183917</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>16.51488322964522</v>
+        <v>9.892033945605846</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.7184838271385681</v>
+        <v>0.2346939174278734</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L93" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M93" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-29.68679364770203</v>
+        <v>-0.1126878788656517</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6405</v>
+        <v>6442</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>悅城</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>369.9722397214716</v>
+        <v>372.1757267281355</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>55.7</v>
+        <v>1480</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,25 +5428,25 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.01916308595516</v>
+        <v>35.11839568595813</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.22245864259789</v>
+        <v>16.51488322964522</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1.003596055848556</v>
+        <v>0.7184838271385681</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M94" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-1.356099503572069</v>
+        <v>-29.68679364770203</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5456,21 +5456,21 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6230</v>
+        <v>6405</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>悅城</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>360.1325994701953</v>
+        <v>369.9722397214716</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>124</v>
+        <v>55.7</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>40.59913532017764</v>
+        <v>40.01916308595516</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>17.3253221750114</v>
+        <v>17.22245864259789</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.4545134327616</v>
+        <v>1.003596055848556</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0061754275391461</v>
+        <v>-1.356099503572069</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6164</v>
+        <v>6225</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>華興</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>359.9481550569465</v>
+        <v>362.9006456083451</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>14.95</v>
+        <v>23.3</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>56.66915190676168</v>
+        <v>51.86622281759339</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>25.98464873145076</v>
+        <v>11.41918567163419</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.8948155056946507</v>
+        <v>0.2609126346787915</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,11 +5552,11 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1312034857149905</v>
+        <v>0.2546357645545872</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6183</v>
+        <v>6230</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>關貿</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>312.3171488900049</v>
+        <v>320.1325994701953</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>90.2</v>
+        <v>124</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>50.01018323720761</v>
+        <v>40.59913532017764</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.6175530211043</v>
+        <v>17.3253221750114</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.4177160957473697</v>
+        <v>0.4545134327616</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,11 +5870,11 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.1336516835633102</v>
+        <v>-0.0061754275391461</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6205</v>
+        <v>6183</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>詮欣</t>
+          <t>關貿</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>265.2735408537372</v>
+        <v>272.3171488900049</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>69.5</v>
+        <v>90.2</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>38.85740384461294</v>
+        <v>50.01018323720761</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>12.11675972137562</v>
+        <v>14.6175530211043</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.4856730437017876</v>
+        <v>0.4177160957473697</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,48 +6241,48 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.8315558906184639</v>
+        <v>0.1336516835633102</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6287</v>
+        <v>6205</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>元隆</t>
+          <t>詮欣</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>260.3181940124887</v>
+        <v>265.2735408537372</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>8.890000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2025-06-20</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G110" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>83.95649937448576</v>
+        <v>38.85740384461294</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v/>
+        <v>12.11675972137562</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.3819364013941486</v>
+        <v>0.4856730437017876</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,48 +6294,48 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0010410561976055</v>
+        <v>-0.8315558906184639</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6485</v>
+        <v>6287</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>點序</t>
+          <t>元隆</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>256.3276120391334</v>
+        <v>260.3181940124887</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>76.8</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2025-06-20</t>
         </is>
       </c>
       <c r="G111" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>34.16736105001425</v>
+        <v>83.95649937448576</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.51448012328121</v>
+        <v/>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4515810770101136</v>
+        <v>0.3819364013941486</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.61158523585227</v>
+        <v>-0.0010410561976055</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, rsi_strong, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6224</v>
+        <v>6485</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>聚鼎</t>
+          <t>點序</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>235.7833834298944</v>
+        <v>256.3276120391334</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>74.5</v>
+        <v>76.8</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.01206228379726</v>
+        <v>34.16736105001425</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.96568693024997</v>
+        <v>18.51448012328121</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.330447438587333</v>
+        <v>0.4515810770101136</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.6992786951734105</v>
+        <v>-0.61158523585227</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6443</v>
+        <v>6224</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>元晶</t>
+          <t>聚鼎</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>223.0431284062792</v>
+        <v>235.7833834298944</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>31.25</v>
+        <v>74.5</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>29.60682074951428</v>
+        <v>46.01206228379726</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>19.1329754266465</v>
+        <v>14.96568693024997</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3876295332244988</v>
+        <v>0.330447438587333</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.5117537067478808</v>
+        <v>-0.6992786951734105</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6463,21 +6463,21 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6269</v>
+        <v>6443</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>台郡</t>
+          <t>元晶</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>211.7835147193647</v>
+        <v>223.0431284062792</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>62.5</v>
+        <v>31.25</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>41.10985930204327</v>
+        <v>29.60682074951428</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.98375080325065</v>
+        <v>19.1329754266465</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.2327752866704111</v>
+        <v>0.3876295332244988</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-1.713790328727013</v>
+        <v>-0.5117537067478808</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,52 +6516,105 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
+        <v>6269</v>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>台郡</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>211.7835147193647</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>41.10985930204327</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>17.98375080325065</v>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>0.2327752866704111</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N115" s="2" t="n">
+        <v>-1.713790328727013</v>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
         <v>6236</v>
       </c>
-      <c r="B115" s="2" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>中湛</t>
         </is>
       </c>
-      <c r="C115" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D115" s="2" t="n">
+      <c r="C116" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="2" t="n">
         <v>149</v>
       </c>
-      <c r="E115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H115" s="2" t="n">
+      <c r="E116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
         <v>48.11588819305965</v>
       </c>
-      <c r="I115" s="2" t="n">
+      <c r="I116" s="2" t="n">
         <v>7.81431113047173</v>
       </c>
-      <c r="J115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M115" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N115" s="2" t="n">
+      <c r="J116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N116" s="2" t="n">
         <v>0.100536975472327</v>
       </c>
-      <c r="O115" s="2" t="inlineStr">
+      <c r="O116" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, obv_uptrend</t>
         </is>

</xml_diff>

<commit_message>
scan: seg5 2026-07-10 20:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq6_2026-07-09.xlsx
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1136.488689421495</v>
+        <v>1156.488689421495</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>73.3</v>
@@ -633,21 +633,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>6416</v>
+        <v>6214</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>精誠</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>979.3786316376716</v>
+        <v>999.071936332872</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>143.5</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>76.06429831862002</v>
+        <v>60.50422918684576</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>25.63228320159281</v>
+        <v>17.0889865435334</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>3.537863163767159</v>
+        <v>2.433126022514748</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -676,31 +676,31 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>2.003064935013459</v>
+        <v>0.3179615362093037</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, cci_momentum, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>6257</v>
+        <v>6416</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>961.4087282385286</v>
+        <v>979.3786316376716</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>244.5</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,49 +711,49 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55.05093771502047</v>
+        <v>76.06429831862002</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>23.26007460439195</v>
+        <v>25.63228320159281</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.5128257206867946</v>
+        <v>3.537863163767159</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.3007865075158751</v>
+        <v>2.003064935013459</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>6214</v>
+        <v>6257</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>精誠</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>959.0719363328718</v>
+        <v>961.4087282385286</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>143.5</v>
+        <v>244.5</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,29 +764,29 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>60.50422918684576</v>
+        <v>55.05093771502047</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>17.0889865435334</v>
+        <v>23.26007460439195</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>2.433126022514748</v>
+        <v>0.5128257206867946</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.3179615362093037</v>
+        <v>0.3007865075158751</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, cci_momentum, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -951,21 +951,21 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6270</v>
+        <v>6213</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>倍微</t>
+          <t>聯茂</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>903.4944641918446</v>
+        <v>918.2917432855902</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>38.1</v>
+        <v>385</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,49 +976,49 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>56.16803427596305</v>
+        <v>66.52584889707384</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>45.41071668250792</v>
+        <v>27.52381890203836</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.9385230014741648</v>
+        <v>1.258419360207691</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.6488655822336251</v>
+        <v>5.515810684032736</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6477</v>
+        <v>6270</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>安集</t>
+          <t>倍微</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>900.5984959459859</v>
+        <v>903.4944641918446</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>39.85</v>
+        <v>38.1</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,16 +1029,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>64.36310514047798</v>
+        <v>56.16803427596305</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>22.21366084951176</v>
+        <v>45.41071668250792</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>3.159849594598582</v>
+        <v>0.9385230014741648</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.8494610209375359</v>
+        <v>-0.6488655822336251</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6213</v>
+        <v>6477</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>聯茂</t>
+          <t>安集</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>878.2917432855902</v>
+        <v>900.5984959459859</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>385</v>
+        <v>39.85</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,49 +1082,49 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>66.52584889707384</v>
+        <v>64.36310514047798</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>27.52381890203836</v>
+        <v>22.21366084951176</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1.258419360207691</v>
+        <v>3.159849594598582</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>5.515810684032736</v>
+        <v>0.8494610209375359</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6282</v>
+        <v>6197</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>康舒</t>
+          <t>佳必琪</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>815.1661862649786</v>
+        <v>828.220035793717</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>57.6</v>
+        <v>358.5</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,49 +1135,49 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>48.98349110842224</v>
+        <v>58.69446535738361</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>23.21749066799558</v>
+        <v>40.89797096720127</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.9926387085112316</v>
+        <v>0.8309268861561855</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M13" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.2461605351610881</v>
+        <v>-3.042639085888481</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>6241</v>
+        <v>6282</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>鑫永洋</t>
+          <t>康舒</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>813.0398195169184</v>
+        <v>815.1661862649786</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>15.75</v>
+        <v>57.6</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,49 +1188,49 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>67.91588948480008</v>
+        <v>48.98349110842224</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>42.29721981571507</v>
+        <v>23.21749066799558</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.7893554100046339</v>
+        <v>0.9926387085112316</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M14" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-0.0514089759588609</v>
+        <v>-0.2461605351610881</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6414</v>
+        <v>6241</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>鑫永洋</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>803.458074698501</v>
+        <v>813.0398195169184</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>394</v>
+        <v>15.75</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,16 +1241,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59.35973158644198</v>
+        <v>67.91588948480008</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>19.92414366320097</v>
+        <v>42.29721981571507</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1.18854989594806</v>
+        <v>0.7893554100046339</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>1.700399767192037</v>
+        <v>-0.0514089759588609</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6197</v>
+        <v>6414</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>佳必琪</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>788.220035793717</v>
+        <v>803.458074698501</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>358.5</v>
+        <v>394</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,29 +1294,29 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>58.69446535738361</v>
+        <v>59.35973158644198</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>40.89797096720127</v>
+        <v>19.92414366320097</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.8309268861561855</v>
+        <v>1.18854989594806</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-3.042639085888481</v>
+        <v>1.700399767192037</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1481,21 +1481,21 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6285</v>
+        <v>6209</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>今國光</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>740.1824626219473</v>
+        <v>743.8443291860746</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>260.5</v>
+        <v>80.8</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,49 +1506,49 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>49.66126258135844</v>
+        <v>48.67482667949162</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>17.42376200502451</v>
+        <v>26.55887681155335</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>2.043911053938038</v>
+        <v>0.4540819283646607</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.0247863523021827</v>
+        <v>-1.372872544755097</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6259</v>
+        <v>6285</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>百徽</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>734.2079347452019</v>
+        <v>740.1824626219473</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>38.45</v>
+        <v>260.5</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,49 +1559,49 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>56.71933780594453</v>
+        <v>49.66126258135844</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>37.27624546620987</v>
+        <v>17.42376200502451</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.6456519025936032</v>
+        <v>2.043911053938038</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.150824480299021</v>
+        <v>0.0247863523021827</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6417</v>
+        <v>6259</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>韋僑</t>
+          <t>百徽</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>715.7846223339815</v>
+        <v>734.2079347452019</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>135.5</v>
+        <v>38.45</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>55.29641028056212</v>
+        <v>56.71933780594453</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>10.87399987697184</v>
+        <v>37.27624546620987</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.4525698906929652</v>
+        <v>0.6456519025936032</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.366861573603427</v>
+        <v>-0.150824480299021</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6185</v>
+        <v>6417</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>幃翔</t>
+          <t>韋僑</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>710.111078177459</v>
+        <v>715.7846223339815</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>14.5</v>
+        <v>135.5</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>54.46539144255123</v>
+        <v>55.29641028056212</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>20.49066768291864</v>
+        <v>10.87399987697184</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.8739787087878066</v>
+        <v>0.4525698906929652</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.0014006804678929</v>
+        <v>0.366861573603427</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6209</v>
+        <v>6185</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>幃翔</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>703.8443291860746</v>
+        <v>710.111078177459</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>80.8</v>
+        <v>14.5</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>48.67482667949162</v>
+        <v>54.46539144255123</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>26.55887681155335</v>
+        <v>20.49066768291864</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.4540819283646607</v>
+        <v>0.8739787087878066</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,11 +1736,11 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-1.372872544755097</v>
+        <v>-0.0014006804678929</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2064,21 +2064,21 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6176</v>
+        <v>6175</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>630.7227281970102</v>
+        <v>630.7023836445761</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>90.59999999999999</v>
+        <v>105</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>45.95921703984428</v>
+        <v>50.64811739707996</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>18.23336187973892</v>
+        <v>35.94163140743942</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.4865562411329991</v>
+        <v>0.3016672626794371</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.7301936113755336</v>
+        <v>-1.732389440968922</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6175</v>
+        <v>6271</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>630.7023836445761</v>
+        <v>621.0928621229963</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>105</v>
+        <v>252</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>50.64811739707996</v>
+        <v>51.19847872710957</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>35.94163140743942</v>
+        <v>24.45229549813269</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.3016672626794371</v>
+        <v>0.5346225556122013</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-1.732389440968922</v>
+        <v>-2.368416313269387</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6271</v>
+        <v>6187</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>萬潤</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>621.0928621229963</v>
+        <v>612.8943797335932</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>252</v>
+        <v>1050</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,49 +2195,49 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>51.19847872710957</v>
+        <v>48.66755686619767</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>24.45229549813269</v>
+        <v>10.93429019971599</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.5346225556122013</v>
+        <v>1.418708493139663</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-2.368416313269387</v>
+        <v>-8.324338563349585</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6187</v>
+        <v>6204</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>萬潤</t>
+          <t>艾華</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>612.8943797335932</v>
+        <v>604.8897832036441</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1050</v>
+        <v>98.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,49 +2248,49 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>48.66755686619767</v>
+        <v>41.48366736939177</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>10.93429019971599</v>
+        <v>28.33411598523973</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.418708493139663</v>
+        <v>0.4866331027247718</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-8.324338563349585</v>
+        <v>-3.300467962525275</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6204</v>
+        <v>6196</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>艾華</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>604.8897832036441</v>
+        <v>600.7545257562992</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>98.5</v>
+        <v>549</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>41.48366736939177</v>
+        <v>54.08532215887169</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>28.33411598523973</v>
+        <v>28.05357859083168</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.4866331027247718</v>
+        <v>0.8671349625130681</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>1</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-3.300467962525275</v>
+        <v>-5.07453997068513</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2329,21 +2329,21 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6207</v>
+        <v>6176</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>雷科</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>600.1406899368378</v>
+        <v>600.7227281970102</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>144</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>53.18377042450608</v>
+        <v>45.95921703984428</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>45.32246469824553</v>
+        <v>18.23336187973892</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.6027701256140928</v>
+        <v>0.4865562411329991</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-4.07561757387931</v>
+        <v>0.7301936113755336</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6423</v>
+        <v>6207</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>億而得-創</t>
+          <t>雷科</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>598.2649519596628</v>
+        <v>600.1406899368378</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>87.5</v>
+        <v>144</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>52.78562191561644</v>
+        <v>53.18377042450608</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>24.05886629173131</v>
+        <v>45.32246469824553</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.449606935936577</v>
+        <v>0.6027701256140928</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1.391202298523601</v>
+        <v>-4.07561757387931</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6411</v>
+        <v>6423</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>晶焱</t>
+          <t>億而得-創</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>598.185288820585</v>
+        <v>598.2649519596628</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>97</v>
+        <v>87.5</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>48.65597037531157</v>
+        <v>52.78562191561644</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>23.89270650366059</v>
+        <v>24.05886629173131</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.3075844162237828</v>
+        <v>1.449606935936577</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.9486744607386286</v>
+        <v>1.391202298523601</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6432</v>
+        <v>6411</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>今展科</t>
+          <t>晶焱</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>598.0981413944291</v>
+        <v>598.185288820585</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>75.59999999999999</v>
+        <v>97</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>53.70575596736259</v>
+        <v>48.65597037531157</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>30.79813657649377</v>
+        <v>23.89270650366059</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.4540777874413215</v>
+        <v>0.3075844162237828</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-1.030026691637948</v>
+        <v>-0.9486744607386286</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6472</v>
+        <v>6432</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>保瑞</t>
+          <t>今展科</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>597.2762653443908</v>
+        <v>598.0981413944291</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>426</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.9033810100284</v>
+        <v>53.70575596736259</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>30.53533734636597</v>
+        <v>30.79813657649377</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.6494925873039354</v>
+        <v>0.4540777874413215</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.8607435001690007</v>
+        <v>-1.030026691637948</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6449</v>
+        <v>6472</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>鈺邦</t>
+          <t>保瑞</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>591.2268070754961</v>
+        <v>597.2762653443908</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>352</v>
+        <v>426</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>50.76819919769214</v>
+        <v>54.9033810100284</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>20.47720114184548</v>
+        <v>30.53533734636597</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.9009453855020156</v>
+        <v>0.6494925873039354</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-9.52114033297195</v>
+        <v>-0.8607435001690007</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6266</v>
+        <v>6449</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>泰詠</t>
+          <t>鈺邦</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>590.4762477089753</v>
+        <v>591.2268070754961</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>25.3</v>
+        <v>352</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>42.41054686377194</v>
+        <v>50.76819919769214</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>19.56985632431543</v>
+        <v>20.47720114184548</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.6037582883223328</v>
+        <v>0.9009453855020156</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.0660213803907002</v>
+        <v>-9.52114033297195</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6245</v>
+        <v>6266</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>立端</t>
+          <t>泰詠</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>590.004126024571</v>
+        <v>590.4762477089753</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>80.8</v>
+        <v>25.3</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>47.58552239867173</v>
+        <v>42.41054686377194</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>11.85395500569073</v>
+        <v>19.56985632431543</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.7176929893924647</v>
+        <v>0.6037582883223328</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0872110605998839</v>
+        <v>0.0660213803907002</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6435</v>
+        <v>6245</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>大中</t>
+          <t>立端</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>576.1851267043151</v>
+        <v>590.004126024571</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>375</v>
+        <v>80.8</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>60.02396593640601</v>
+        <v>47.58552239867173</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>35.11373582234368</v>
+        <v>11.85395500569073</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.800487862173044</v>
+        <v>0.7176929893924647</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1.27326385425064</v>
+        <v>0.0872110605998839</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6465</v>
+        <v>6166</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>威潤</t>
+          <t>凌華</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>575.1809853817028</v>
+        <v>589.6703293062818</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>63.3</v>
+        <v>134.5</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>56.1046732562139</v>
+        <v>50.95900459453849</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>26.27029971801192</v>
+        <v>37.25304903070406</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.753080817871749</v>
+        <v>0.6481348291603305</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-1.136157175014425</v>
+        <v>-2.634043287392596</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6208</v>
+        <v>6165</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>日揚</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>574.229836358609</v>
+        <v>589.5856464879407</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>90.3</v>
+        <v>50.1</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>47.39148571270285</v>
+        <v>55.89803805348778</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>15.45204016428327</v>
+        <v>20.28593810246351</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.1722180031841522</v>
+        <v>1.049333799631696</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.225666944879956</v>
+        <v>0.3791670455581503</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6239</v>
+        <v>6435</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>大中</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>573.9125542434286</v>
+        <v>576.1851267043151</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,49 +2937,49 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>48.44503578764906</v>
+        <v>60.02396593640601</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>23.80075786039455</v>
+        <v>35.11373582234368</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.3459569826215111</v>
+        <v>0.800487862173044</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-4.586864459811611</v>
+        <v>1.27326385425064</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6165</v>
+        <v>6465</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>威潤</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>569.5856464879407</v>
+        <v>575.1809853817028</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>50.1</v>
+        <v>63.3</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>55.89803805348778</v>
+        <v>56.1046732562139</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>20.28593810246351</v>
+        <v>26.27029971801192</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.049333799631696</v>
+        <v>0.753080817871749</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.3791670455581503</v>
+        <v>-1.136157175014425</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6235</v>
+        <v>6208</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>華孚</t>
+          <t>日揚</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>564.7068725170659</v>
+        <v>574.229836358609</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>42.4</v>
+        <v>90.3</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>50.95768947600303</v>
+        <v>47.39148571270285</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>20.46692171898411</v>
+        <v>15.45204016428327</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.042148858262224</v>
+        <v>0.1722180031841522</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.4104142795117735</v>
+        <v>-1.225666944879956</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6196</v>
+        <v>6239</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>560.7545257562992</v>
+        <v>573.9125542434286</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>549</v>
+        <v>320</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,49 +3096,49 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>54.08532215887169</v>
+        <v>48.44503578764906</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>28.05357859083168</v>
+        <v>23.80075786039455</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.8671349625130681</v>
+        <v>0.3459569826215111</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M50" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-5.07453997068513</v>
+        <v>-4.586864459811611</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6166</v>
+        <v>6235</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>凌華</t>
+          <t>華孚</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>549.6703293062818</v>
+        <v>564.7068725170659</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>134.5</v>
+        <v>42.4</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>50.95900459453849</v>
+        <v>50.95768947600303</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>37.25304903070406</v>
+        <v>20.46692171898411</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.6481348291603305</v>
+        <v>1.042148858262224</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-2.634043287392596</v>
+        <v>0.4104142795117735</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6220</v>
+        <v>6206</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>岳豐</t>
+          <t>飛捷</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>544.427599966453</v>
+        <v>557.206889349207</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>33.6</v>
+        <v>131.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46.02052274010901</v>
+        <v>50.80161092657132</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>36.82475523537035</v>
+        <v>11.05857041742693</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.1265911095062542</v>
+        <v>1.596155571684044</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.4648632195580982</v>
+        <v>0.1683190083713577</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6261</v>
+        <v>6220</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>岳豐</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>539.7984202187615</v>
+        <v>544.427599966453</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>33.6</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>39.89966499434699</v>
+        <v>46.02052274010901</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>17.70217002504111</v>
+        <v>36.82475523537035</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.3258076319138756</v>
+        <v>0.1265911095062542</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.0227109598430041</v>
+        <v>-0.4648632195580982</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6173</v>
+        <v>6189</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>信昌電</t>
+          <t>豐藝</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>526.9722281302035</v>
+        <v>543.1171308580567</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>275</v>
+        <v>50.4</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>50.18098418175746</v>
+        <v>44.42019512273473</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>26.82029344258599</v>
+        <v>18.72534459086502</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.056435950495918</v>
+        <v>0.2994648258745055</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-8.545329832583654</v>
+        <v>-0.32970209837375</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6189</v>
+        <v>6261</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>豐藝</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>523.1171308580568</v>
+        <v>539.7984202187615</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>50.4</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>44.42019512273473</v>
+        <v>39.89966499434699</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.72534459086502</v>
+        <v>17.70217002504111</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.2994648258745055</v>
+        <v>0.3258076319138756</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.32970209837375</v>
+        <v>-0.0227109598430041</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6192</v>
+        <v>6215</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>和椿</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>522.7966888452497</v>
+        <v>528.0668217122557</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>120</v>
+        <v>113.5</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46.57038285186782</v>
+        <v>51.95973173451051</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>19.77975771667846</v>
+        <v>17.62415730350409</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2885966311380484</v>
+        <v>0.944676363510302</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1031038247129059</v>
+        <v>1.398526045593522</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6206</v>
+        <v>6173</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>飛捷</t>
+          <t>信昌電</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>517.206889349207</v>
+        <v>526.9722281302035</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>131.5</v>
+        <v>275</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>50.80161092657132</v>
+        <v>50.18098418175746</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>11.05857041742693</v>
+        <v>26.82029344258599</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>1.596155571684044</v>
+        <v>1.056435950495918</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1683190083713577</v>
+        <v>-8.545329832583654</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6216</v>
+        <v>6228</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>509.7726759338609</v>
+        <v>505.2527726489098</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>23.15</v>
+        <v>19.1</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>52.51581439552675</v>
+        <v>44.66734659846346</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>12.02130481601512</v>
+        <v>4.744489874638209</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.6623511287610836</v>
+        <v>0.1213040586205195</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.05811366871442</v>
+        <v>-0.0666148916581248</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6228</v>
+        <v>6244</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>全譜</t>
+          <t>茂迪</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>505.2527726489098</v>
+        <v>503.2552975876344</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>19.1</v>
+        <v>27</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.66734659846346</v>
+        <v>45.56871279071334</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>4.744489874638209</v>
+        <v>10.21266174976934</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.1213040586205195</v>
+        <v>0.2920367732268786</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0666148916581248</v>
+        <v>-0.0648959710707384</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6244</v>
+        <v>6277</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>茂迪</t>
+          <t>宏正</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>503.2552975876344</v>
+        <v>498.0865178878039</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>27</v>
+        <v>70.7</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>45.56871279071334</v>
+        <v>44.52558862040208</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>10.21266174976934</v>
+        <v>26.28544254631901</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.2920367732268786</v>
+        <v>0.6633441183231713</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0648959710707384</v>
+        <v>-0.0103847418663265</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6277</v>
+        <v>6192</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>宏正</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>498.0865178878039</v>
+        <v>492.7966888452498</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>70.7</v>
+        <v>120</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>44.52558862040208</v>
+        <v>46.57038285186782</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>26.28544254631901</v>
+        <v>19.77975771667846</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.6633441183231713</v>
+        <v>0.2885966311380484</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>1</v>
@@ -3697,11 +3697,11 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0103847418663265</v>
+        <v>0.1031038247129059</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -3760,21 +3760,21 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6215</v>
+        <v>6216</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>和椿</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>488.0668217122557</v>
+        <v>479.7726759338609</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>113.5</v>
+        <v>23.15</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>51.95973173451051</v>
+        <v>52.51581439552675</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>17.62415730350409</v>
+        <v>12.02130481601512</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.944676363510302</v>
+        <v>0.6623511287610836</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,11 +3803,11 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.398526045593522</v>
+        <v>0.05811366871442</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -3919,21 +3919,21 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6451</v>
+        <v>6168</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>宏齊</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>460.5090043333418</v>
+        <v>463.7828326677232</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>518</v>
+        <v>28.85</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>45.18548299802012</v>
+        <v>48.91567536944652</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>20.61927913671785</v>
+        <v>23.86009076031464</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.6043869457439386</v>
+        <v>0.5031973367918018</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-9.507617469249002</v>
+        <v>-0.2869513207650043</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6233</v>
+        <v>6451</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>旺玖</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>456.3786575160711</v>
+        <v>460.5090043333418</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>24.7</v>
+        <v>518</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>46.6303197746648</v>
+        <v>45.18548299802012</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.32643744125292</v>
+        <v>20.61927913671785</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.6120290265707217</v>
+        <v>0.6043869457439386</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.0415921231305314</v>
+        <v>-9.507617469249002</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6274</v>
+        <v>6233</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>旺玖</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>455.3358416368599</v>
+        <v>456.3786575160711</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>1570</v>
+        <v>24.7</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>48.09520288082244</v>
+        <v>46.6303197746648</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>23.795092210229</v>
+        <v>11.32643744125292</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.8056576367210952</v>
+        <v>0.6120290265707217</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-25.50789987085458</v>
+        <v>-0.0415921231305314</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6203</v>
+        <v>6274</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>海韻電</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>453.8863334868984</v>
+        <v>455.3358416368599</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>67.2</v>
+        <v>1570</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.57966392410312</v>
+        <v>48.09520288082244</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.10053069941169</v>
+        <v>23.795092210229</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.4463445108126535</v>
+        <v>0.8056576367210952</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.1150095001022786</v>
+        <v>-25.50789987085458</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6234</v>
+        <v>6203</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>高僑</t>
+          <t>海韻電</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>453.3924442741192</v>
+        <v>453.8863334868984</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>42.2</v>
+        <v>67.2</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>42.26779425829178</v>
+        <v>46.57966392410312</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>13.05855607056404</v>
+        <v>15.10053069941169</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.996817213305069</v>
+        <v>0.4463445108126535</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.2247701788352369</v>
+        <v>0.1150095001022786</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6281</v>
+        <v>6234</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>全國電</t>
+          <t>高僑</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>449.3342376270039</v>
+        <v>453.3924442741192</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>52</v>
+        <v>42.2</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>56.62625250920745</v>
+        <v>42.26779425829178</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.92313951576784</v>
+        <v>13.05855607056404</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4672738782129317</v>
+        <v>0.996817213305069</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.0802573539408627</v>
+        <v>-0.2247701788352369</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6168</v>
+        <v>6281</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>宏齊</t>
+          <t>全國電</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>443.7828326677232</v>
+        <v>449.3342376270039</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>28.85</v>
+        <v>52</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.91567536944652</v>
+        <v>56.62625250920745</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>23.86009076031464</v>
+        <v>12.92313951576784</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.5031973367918018</v>
+        <v>0.4672738782129317</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,11 +4280,11 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.2869513207650043</v>
+        <v>0.0802573539408627</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -4396,18 +4396,18 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6201</v>
+        <v>6470</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>宇智</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>429.3913444803261</v>
+        <v>428.6954580025336</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>48.2</v>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>47.25179204900812</v>
+        <v>43.87120259228157</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>12.91561406465129</v>
+        <v>10.7933361805923</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.7091451287235034</v>
+        <v>0.2870718049139532</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.07570005957403431</v>
+        <v>-0.1652794096263817</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6470</v>
+        <v>6177</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>宇智</t>
+          <t>達麗</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>428.6954580025336</v>
+        <v>425.9484505658648</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>48.2</v>
+        <v>45.3</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>43.87120259228157</v>
+        <v>47.57489387764495</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>10.7933361805923</v>
+        <v>18.49489665722346</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.2870718049139532</v>
+        <v>0.2200969188721565</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1652794096263817</v>
+        <v>-0.1489141335302252</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6177</v>
+        <v>6237</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>達麗</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>425.9484505658648</v>
+        <v>424.5636897177679</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>45.3</v>
+        <v>42</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>47.57489387764495</v>
+        <v>39.47391672999221</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>18.49489665722346</v>
+        <v>15.33426235374559</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.2200969188721565</v>
+        <v>0.3681852680468525</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.1489141335302252</v>
+        <v>-0.4402223312269442</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6237</v>
+        <v>6218</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>424.5636897177679</v>
+        <v>423.5998250586194</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>42</v>
+        <v>37.65</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>39.47391672999221</v>
+        <v>53.71863566754495</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>15.33426235374559</v>
+        <v>12.11336053714617</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.3681852680468525</v>
+        <v>0.7799099700886115</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.4402223312269442</v>
+        <v>-0.0765627468007149</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6218</v>
+        <v>6438</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>423.5998250586194</v>
+        <v>420.9571224619286</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>37.65</v>
+        <v>150</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>53.71863566754495</v>
+        <v>42.43657643210879</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>12.11336053714617</v>
+        <v>18.95269682823951</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.7799099700886115</v>
+        <v>0.355053965030203</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0765627468007149</v>
+        <v>0.0937697190638255</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6438</v>
+        <v>6184</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>大豐電</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>420.9571224619286</v>
+        <v>420.1887932823112</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>150</v>
+        <v>42.95</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.43657643210879</v>
+        <v>23.08460877876179</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>18.95269682823951</v>
+        <v>34.84741265862615</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.355053965030203</v>
+        <v>0.3583230749555412</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0937697190638255</v>
+        <v>-0.164233773995498</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6184</v>
+        <v>6190</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>大豐電</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>420.1887932823112</v>
+        <v>418.9408680563363</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>42.95</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>23.08460877876179</v>
+        <v>50.34237102418618</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>34.84741265862615</v>
+        <v>15.63189548975667</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.3583230749555412</v>
+        <v>0.4859050337067814</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.164233773995498</v>
+        <v>-0.2071625297881087</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6190</v>
+        <v>6167</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>418.9408680563363</v>
+        <v>418.1672673971372</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>82.09999999999999</v>
+        <v>11.95</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>50.34237102418618</v>
+        <v>48.06859488036503</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>15.63189548975667</v>
+        <v>12.51517199083887</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.4859050337067814</v>
+        <v>0.3064617242987439</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2071625297881087</v>
+        <v>-3.267974353826641e-05</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6167</v>
+        <v>6191</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>418.1672673971372</v>
+        <v>417.6157292145597</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>11.95</v>
+        <v>101</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>48.06859488036503</v>
+        <v>48.80069786817602</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.51517199083887</v>
+        <v>27.93277159754891</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.3064617242987439</v>
+        <v>0.4765533747053406</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-3.267974353826641e-05</v>
+        <v>-0.0634150839392706</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6191</v>
+        <v>6198</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>瑞築</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>417.6157292145597</v>
+        <v>410.9554246216042</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>101</v>
+        <v>20.35</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.80069786817602</v>
+        <v>50.12740667423494</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>27.93277159754891</v>
+        <v>7.069923903668688</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.4765533747053406</v>
+        <v>0.4026442608430207</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0634150839392706</v>
+        <v>0.0011358756227049</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6198</v>
+        <v>6291</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>410.9554246216042</v>
+        <v>405.8446327600136</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>20.35</v>
+        <v>463.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,49 +4951,49 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>50.12740667423494</v>
+        <v>40.12907838236885</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>7.069923903668688</v>
+        <v>15.65361422755754</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.4026442608430207</v>
+        <v>0.6961864646384438</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M85" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0011358756227049</v>
+        <v>-15.20329251158969</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6291</v>
+        <v>6278</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>405.8446327600136</v>
+        <v>404.0760437863103</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>463.5</v>
+        <v>199.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,49 +5004,49 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>40.12907838236885</v>
+        <v>47.86320449976485</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>15.65361422755754</v>
+        <v>16.013163606553</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.6961864646384438</v>
+        <v>0.9402907544968636</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M86" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-15.20329251158969</v>
+        <v>-1.130259753047042</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6278</v>
+        <v>6225</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>404.0760437863103</v>
+        <v>402.9006456083451</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>199.5</v>
+        <v>23.3</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,29 +5057,29 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>47.86320449976485</v>
+        <v>51.86622281759339</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>16.013163606553</v>
+        <v>11.41918567163419</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.9402907544968636</v>
+        <v>0.2609126346787915</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M87" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-1.130259753047042</v>
+        <v>0.2546357645545872</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -5138,21 +5138,21 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6164</v>
+        <v>6201</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>華興</t>
+          <t>亞弘電</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>389.9481550569465</v>
+        <v>399.3913444803261</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>14.95</v>
+        <v>48.2</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>56.66915190676168</v>
+        <v>47.25179204900812</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>25.98464873145076</v>
+        <v>12.91561406465129</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.8948155056946507</v>
+        <v>0.7091451287235034</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,11 +5181,11 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.1312034857149905</v>
+        <v>0.07570005957403431</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -5509,21 +5509,21 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6225</v>
+        <v>6230</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>天瀚</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>362.9006456083451</v>
+        <v>360.1325994701953</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>23.3</v>
+        <v>124</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>51.86622281759339</v>
+        <v>40.59913532017764</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.41918567163419</v>
+        <v>17.3253221750114</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.2609126346787915</v>
+        <v>0.4545134327616</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.2546357645545872</v>
+        <v>-0.0061754275391461</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6222</v>
+        <v>6164</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>立軒</t>
+          <t>華興</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>358.4483792499668</v>
+        <v>359.9481550569465</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>20.9</v>
+        <v>14.95</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>51.40958420165202</v>
+        <v>56.66915190676168</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>22.86729686248819</v>
+        <v>25.98464873145076</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.4855595161245053</v>
+        <v>0.8948155056946507</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0284207246717396</v>
+        <v>0.1312034857149905</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6456</v>
+        <v>6222</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>立軒</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>351.7533575982047</v>
+        <v>358.4483792499668</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>70.7</v>
+        <v>20.9</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>49.13656794039597</v>
+        <v>51.40958420165202</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>16.36721412391648</v>
+        <v>22.86729686248819</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.6778549352853837</v>
+        <v>0.4855595161245053</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.0253771857409628</v>
+        <v>0.0284207246717396</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6290</v>
+        <v>6456</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>良維</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>345.9428538547477</v>
+        <v>351.7533575982047</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>298.5</v>
+        <v>70.7</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>45.56895683047549</v>
+        <v>49.13656794039597</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>9.953207315259752</v>
+        <v>16.36721412391648</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.521055737723002</v>
+        <v>0.6778549352853837</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-1.682989209905118</v>
+        <v>-0.0253771857409628</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6462</v>
+        <v>6290</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>神盾</t>
+          <t>良維</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>337.1752366210359</v>
+        <v>345.9428538547477</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>110.5</v>
+        <v>298.5</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>41.38131922642528</v>
+        <v>45.56895683047549</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.55498262897279</v>
+        <v>9.953207315259752</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.2660460997613548</v>
+        <v>0.521055737723002</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.4486174139132075</v>
+        <v>-1.682989209905118</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6170</v>
+        <v>6462</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>統振</t>
+          <t>神盾</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>333.4209710328146</v>
+        <v>337.1752366210359</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>47.25</v>
+        <v>110.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>24.09267480749578</v>
+        <v>41.38131922642528</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>20.12571709646378</v>
+        <v>14.55498262897279</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1.545157345409195</v>
+        <v>0.2660460997613548</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.520097425558904</v>
+        <v>-0.4486174139132075</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6230</v>
+        <v>6170</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>統振</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>320.1325994701953</v>
+        <v>333.4209710328146</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>124</v>
+        <v>47.25</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>40.59913532017764</v>
+        <v>24.09267480749578</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.3253221750114</v>
+        <v>20.12571709646378</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.4545134327616</v>
+        <v>1.545157345409195</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0061754275391461</v>
+        <v>-0.520097425558904</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6283</v>
+        <v>6183</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>淳安</t>
+          <t>關貿</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>310.3954795456821</v>
+        <v>312.3171488900049</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>23.2</v>
+        <v>90.2</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>44.17505451173921</v>
+        <v>50.01018323720761</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>11.66906124171542</v>
+        <v>14.6175530211043</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.2818476029166994</v>
+        <v>0.4177160957473697</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0491292026521335</v>
+        <v>0.1336516835633102</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6194</v>
+        <v>6283</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>育富</t>
+          <t>淳安</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>307.5406268376613</v>
+        <v>310.3954795456821</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>31.8</v>
+        <v>23.2</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>39.25018383417692</v>
+        <v>44.17505451173921</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>12.04318924695395</v>
+        <v>11.66906124171542</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.3230060102340865</v>
+        <v>0.2818476029166994</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.021661772156045</v>
+        <v>-0.0491292026521335</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6441</v>
+        <v>6194</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>廣錠</t>
+          <t>育富</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>297.6005510753579</v>
+        <v>307.5406268376613</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>23</v>
+        <v>31.8</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.97454678888006</v>
+        <v>39.25018383417692</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>12.42262871584943</v>
+        <v>12.04318924695395</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3451211735829833</v>
+        <v>0.3230060102340865</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.1267217425500511</v>
+        <v>-0.021661772156045</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6276</v>
+        <v>6441</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>安鈦克</t>
+          <t>廣錠</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>289.5967295126453</v>
+        <v>297.6005510753579</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>22.1</v>
+        <v>23</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>37.0110540833751</v>
+        <v>49.97454678888006</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>26.08591503497555</v>
+        <v>12.42262871584943</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.3304294516298403</v>
+        <v>0.3451211735829833</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.129017072018742</v>
+        <v>0.1267217425500511</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6415</v>
+        <v>6276</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>安鈦克</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>287.6380987693343</v>
+        <v>289.5967295126453</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>523</v>
+        <v>22.1</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>43.10492316269126</v>
+        <v>37.0110540833751</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18.14980776497181</v>
+        <v>26.08591503497555</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.9135554751610606</v>
+        <v>0.3304294516298403</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-11.60887777007309</v>
+        <v>0.129017072018742</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6412</v>
+        <v>6415</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>277.832624665405</v>
+        <v>287.6380987693343</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>88.8</v>
+        <v>523</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>42.76958212289202</v>
+        <v>43.10492316269126</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>13.43112368097787</v>
+        <v>18.14980776497181</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.3944590485618655</v>
+        <v>0.9135554751610606</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.5983179608620492</v>
+        <v>-11.60887777007309</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6183</v>
+        <v>6412</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>關貿</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>272.3171488900049</v>
+        <v>277.832624665405</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>90.2</v>
+        <v>88.8</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>50.01018323720761</v>
+        <v>42.76958212289202</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>14.6175530211043</v>
+        <v>13.43112368097787</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.4177160957473697</v>
+        <v>0.3944590485618655</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,11 +6241,11 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.1336516835633102</v>
+        <v>-0.5983179608620492</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>